<commit_message>
fixed pipeline to use invoice_timestamp instead of item_timestamp
</commit_message>
<xml_diff>
--- a/pipeline/plugins/manual/_manual_import.xlsx
+++ b/pipeline/plugins/manual/_manual_import.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10808"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24701"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonni/dev/foodsight-backend/pipeline/plugins/manual/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeffe\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B29A18B0-ECB2-6F4F-9DC1-222F2F381872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24EE2317-4F08-41D3-9850-4104B743DF90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39480" yWindow="-5020" windowWidth="35840" windowHeight="20740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2021" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2021'!$A$1:$S$99</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -85,48 +88,21 @@
     <t>Barzahlung</t>
   </si>
   <si>
-    <t>Soda Zitrone</t>
-  </si>
-  <si>
-    <t>Alkoholfreie Getränke</t>
-  </si>
-  <si>
-    <t>Schnitzel</t>
-  </si>
-  <si>
-    <t>Speisen</t>
-  </si>
-  <si>
-    <t>Spaghetti</t>
-  </si>
-  <si>
     <t>08:55:54</t>
   </si>
   <si>
     <t>RG2021/2</t>
   </si>
   <si>
-    <t>Cola</t>
-  </si>
-  <si>
     <t>3132</t>
   </si>
   <si>
-    <t>Worschtsalat</t>
-  </si>
-  <si>
     <t>08:56:02</t>
   </si>
   <si>
     <t>RG2021/3</t>
   </si>
   <si>
-    <t>Cola Bacardi</t>
-  </si>
-  <si>
-    <t>Alkoholische Getränke</t>
-  </si>
-  <si>
     <t>08:56:12</t>
   </si>
   <si>
@@ -157,9 +133,6 @@
     <t>RG2021/8</t>
   </si>
   <si>
-    <t>Spritzer 0,25l</t>
-  </si>
-  <si>
     <t>12:28:54</t>
   </si>
   <si>
@@ -254,17 +227,53 @@
   </si>
   <si>
     <t>Preis</t>
+  </si>
+  <si>
+    <t>Brotware</t>
+  </si>
+  <si>
+    <t>Kürbisbrot</t>
+  </si>
+  <si>
+    <t>Roggen-Mischbrot</t>
+  </si>
+  <si>
+    <t>Baguette</t>
+  </si>
+  <si>
+    <t>Brötchen</t>
+  </si>
+  <si>
+    <t>Sesam-Brötchen</t>
+  </si>
+  <si>
+    <t>Fitness-Brötchen</t>
+  </si>
+  <si>
+    <t>Kuchen</t>
+  </si>
+  <si>
+    <t>Bienenstich</t>
+  </si>
+  <si>
+    <t>Apfelschmandkuchen</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -287,8 +296,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -604,7 +614,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S99"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.8"/>
   <cols>
     <col min="1" max="1" width="25.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
@@ -612,7 +622,7 @@
     <col min="4" max="4" width="17.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="36.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="6.83203125" bestFit="1" customWidth="1"/>
@@ -625,12 +635,12 @@
     <col min="19" max="19" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -672,7 +682,7 @@
         <v>13</v>
       </c>
       <c r="P1" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="Q1" t="s">
         <v>14</v>
@@ -684,7 +694,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -700,11 +710,11 @@
       <c r="E2" t="s">
         <v>20</v>
       </c>
-      <c r="G2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" t="s">
-        <v>22</v>
+      <c r="G2" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -734,7 +744,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -750,11 +760,11 @@
       <c r="E3" t="s">
         <v>20</v>
       </c>
-      <c r="G3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" t="s">
-        <v>22</v>
+      <c r="G3" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -784,7 +794,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -800,11 +810,11 @@
       <c r="E4" t="s">
         <v>20</v>
       </c>
-      <c r="G4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" t="s">
-        <v>24</v>
+      <c r="G4" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -834,7 +844,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -850,11 +860,11 @@
       <c r="E5" t="s">
         <v>20</v>
       </c>
-      <c r="G5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H5" t="s">
-        <v>24</v>
+      <c r="G5" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -884,7 +894,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -892,19 +902,19 @@
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E6" t="s">
         <v>20</v>
       </c>
-      <c r="G6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H6" t="s">
-        <v>22</v>
+      <c r="G6" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -934,7 +944,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -942,19 +952,19 @@
         <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E7" t="s">
         <v>20</v>
       </c>
-      <c r="G7" t="s">
-        <v>25</v>
-      </c>
-      <c r="H7" t="s">
-        <v>24</v>
+      <c r="G7" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -984,7 +994,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -992,22 +1002,22 @@
         <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E8" t="s">
         <v>20</v>
       </c>
       <c r="F8" t="s">
-        <v>29</v>
-      </c>
-      <c r="G8" t="s">
-        <v>30</v>
-      </c>
-      <c r="H8" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J8">
         <v>1</v>
@@ -1037,7 +1047,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -1045,19 +1055,19 @@
         <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E9" t="s">
         <v>20</v>
       </c>
-      <c r="G9" t="s">
-        <v>33</v>
-      </c>
-      <c r="H9" t="s">
-        <v>34</v>
+      <c r="G9" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J9">
         <v>1</v>
@@ -1087,7 +1097,7 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -1095,22 +1105,22 @@
         <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="D10" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E10" t="s">
         <v>20</v>
       </c>
       <c r="F10" t="s">
-        <v>29</v>
-      </c>
-      <c r="G10" t="s">
-        <v>30</v>
-      </c>
-      <c r="H10" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J10">
         <v>1</v>
@@ -1140,7 +1150,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -1148,19 +1158,19 @@
         <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="D11" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="E11" t="s">
         <v>20</v>
       </c>
-      <c r="G11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H11" t="s">
-        <v>22</v>
+      <c r="G11" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J11">
         <v>1</v>
@@ -1190,7 +1200,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -1198,19 +1208,19 @@
         <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="D12" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="E12" t="s">
         <v>20</v>
       </c>
-      <c r="G12" t="s">
-        <v>21</v>
-      </c>
-      <c r="H12" t="s">
-        <v>22</v>
+      <c r="G12" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J12">
         <v>1</v>
@@ -1240,7 +1250,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -1248,19 +1258,19 @@
         <v>17</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="D13" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="E13" t="s">
         <v>20</v>
       </c>
-      <c r="G13" t="s">
-        <v>21</v>
-      </c>
-      <c r="H13" t="s">
-        <v>22</v>
+      <c r="G13" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J13">
         <v>1</v>
@@ -1290,7 +1300,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -1298,19 +1308,19 @@
         <v>17</v>
       </c>
       <c r="C14" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="D14" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="E14" t="s">
         <v>20</v>
       </c>
-      <c r="G14" t="s">
-        <v>21</v>
-      </c>
-      <c r="H14" t="s">
-        <v>22</v>
+      <c r="G14" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J14">
         <v>1</v>
@@ -1340,7 +1350,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -1348,22 +1358,22 @@
         <v>17</v>
       </c>
       <c r="C15" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="D15" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="E15" t="s">
         <v>20</v>
       </c>
       <c r="F15" t="s">
-        <v>29</v>
-      </c>
-      <c r="G15" t="s">
-        <v>30</v>
-      </c>
-      <c r="H15" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J15">
         <v>1</v>
@@ -1393,7 +1403,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -1401,19 +1411,19 @@
         <v>17</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="D16" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="E16" t="s">
         <v>20</v>
       </c>
-      <c r="G16" t="s">
-        <v>25</v>
-      </c>
-      <c r="H16" t="s">
-        <v>24</v>
+      <c r="G16" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J16">
         <v>1</v>
@@ -1443,7 +1453,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -1451,19 +1461,19 @@
         <v>17</v>
       </c>
       <c r="C17" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="D17" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="E17" t="s">
         <v>20</v>
       </c>
-      <c r="G17" t="s">
-        <v>25</v>
-      </c>
-      <c r="H17" t="s">
-        <v>24</v>
+      <c r="G17" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J17">
         <v>1</v>
@@ -1493,7 +1503,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -1501,19 +1511,19 @@
         <v>17</v>
       </c>
       <c r="C18" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="D18" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="E18" t="s">
         <v>20</v>
       </c>
-      <c r="G18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H18" t="s">
-        <v>24</v>
+      <c r="G18" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J18">
         <v>1</v>
@@ -1543,7 +1553,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -1551,19 +1561,19 @@
         <v>17</v>
       </c>
       <c r="C19" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="D19" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="E19" t="s">
         <v>20</v>
       </c>
-      <c r="G19" t="s">
-        <v>21</v>
-      </c>
-      <c r="H19" t="s">
-        <v>22</v>
+      <c r="G19" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J19">
         <v>1</v>
@@ -1593,7 +1603,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -1601,19 +1611,19 @@
         <v>17</v>
       </c>
       <c r="C20" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="D20" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="E20" t="s">
         <v>20</v>
       </c>
-      <c r="G20" t="s">
-        <v>21</v>
-      </c>
-      <c r="H20" t="s">
-        <v>22</v>
+      <c r="G20" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J20">
         <v>1</v>
@@ -1643,7 +1653,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A21" t="s">
         <v>17</v>
       </c>
@@ -1651,19 +1661,19 @@
         <v>17</v>
       </c>
       <c r="C21" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="D21" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="E21" t="s">
         <v>20</v>
       </c>
-      <c r="G21" t="s">
-        <v>28</v>
-      </c>
-      <c r="H21" t="s">
-        <v>22</v>
+      <c r="G21" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J21">
         <v>1</v>
@@ -1693,7 +1703,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A22" t="s">
         <v>17</v>
       </c>
@@ -1701,22 +1711,22 @@
         <v>17</v>
       </c>
       <c r="C22" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="D22" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="E22" t="s">
         <v>20</v>
       </c>
       <c r="F22" t="s">
-        <v>29</v>
-      </c>
-      <c r="G22" t="s">
-        <v>30</v>
-      </c>
-      <c r="H22" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J22">
         <v>1</v>
@@ -1746,7 +1756,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A23" t="s">
         <v>17</v>
       </c>
@@ -1754,22 +1764,22 @@
         <v>17</v>
       </c>
       <c r="C23" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="D23" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="E23" t="s">
         <v>20</v>
       </c>
       <c r="F23" t="s">
-        <v>29</v>
-      </c>
-      <c r="G23" t="s">
-        <v>30</v>
-      </c>
-      <c r="H23" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J23">
         <v>1</v>
@@ -1799,7 +1809,7 @@
         <v>0.48</v>
       </c>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A24" t="s">
         <v>17</v>
       </c>
@@ -1807,19 +1817,19 @@
         <v>17</v>
       </c>
       <c r="C24" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="D24" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="E24" t="s">
         <v>20</v>
       </c>
-      <c r="G24" t="s">
-        <v>21</v>
-      </c>
-      <c r="H24" t="s">
-        <v>22</v>
+      <c r="G24" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J24">
         <v>1</v>
@@ -1849,7 +1859,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A25" t="s">
         <v>17</v>
       </c>
@@ -1857,19 +1867,19 @@
         <v>17</v>
       </c>
       <c r="C25" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="D25" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="E25" t="s">
         <v>20</v>
       </c>
-      <c r="G25" t="s">
-        <v>21</v>
-      </c>
-      <c r="H25" t="s">
-        <v>22</v>
+      <c r="G25" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J25">
         <v>1</v>
@@ -1899,7 +1909,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A26" t="s">
         <v>17</v>
       </c>
@@ -1907,19 +1917,19 @@
         <v>17</v>
       </c>
       <c r="C26" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="D26" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="E26" t="s">
         <v>20</v>
       </c>
-      <c r="G26" t="s">
-        <v>25</v>
-      </c>
-      <c r="H26" t="s">
-        <v>24</v>
+      <c r="G26" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J26">
         <v>1</v>
@@ -1949,7 +1959,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A27" t="s">
         <v>17</v>
       </c>
@@ -1957,19 +1967,19 @@
         <v>17</v>
       </c>
       <c r="C27" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="D27" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="E27" t="s">
         <v>20</v>
       </c>
-      <c r="G27" t="s">
-        <v>25</v>
-      </c>
-      <c r="H27" t="s">
-        <v>24</v>
+      <c r="G27" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J27">
         <v>1</v>
@@ -1999,7 +2009,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A28" t="s">
         <v>17</v>
       </c>
@@ -2007,19 +2017,19 @@
         <v>17</v>
       </c>
       <c r="C28" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="D28" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="E28" t="s">
         <v>20</v>
       </c>
-      <c r="G28" t="s">
-        <v>28</v>
-      </c>
-      <c r="H28" t="s">
-        <v>22</v>
+      <c r="G28" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J28">
         <v>1</v>
@@ -2049,7 +2059,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A29" t="s">
         <v>17</v>
       </c>
@@ -2057,19 +2067,19 @@
         <v>17</v>
       </c>
       <c r="C29" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="D29" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="E29" t="s">
         <v>20</v>
       </c>
-      <c r="G29" t="s">
-        <v>21</v>
-      </c>
-      <c r="H29" t="s">
-        <v>22</v>
+      <c r="G29" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J29">
         <v>1</v>
@@ -2099,7 +2109,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A30" t="s">
         <v>17</v>
       </c>
@@ -2107,19 +2117,19 @@
         <v>17</v>
       </c>
       <c r="C30" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="D30" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="E30" t="s">
         <v>20</v>
       </c>
-      <c r="G30" t="s">
-        <v>21</v>
-      </c>
-      <c r="H30" t="s">
-        <v>22</v>
+      <c r="G30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J30">
         <v>1</v>
@@ -2149,7 +2159,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A31" t="s">
         <v>17</v>
       </c>
@@ -2157,19 +2167,19 @@
         <v>17</v>
       </c>
       <c r="C31" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="D31" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="E31" t="s">
         <v>20</v>
       </c>
-      <c r="G31" t="s">
-        <v>45</v>
-      </c>
-      <c r="H31" t="s">
-        <v>34</v>
+      <c r="G31" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J31">
         <v>1</v>
@@ -2199,7 +2209,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A32" t="s">
         <v>17</v>
       </c>
@@ -2207,19 +2217,19 @@
         <v>17</v>
       </c>
       <c r="C32" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="D32" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="E32" t="s">
         <v>20</v>
       </c>
-      <c r="G32" t="s">
-        <v>23</v>
-      </c>
-      <c r="H32" t="s">
-        <v>24</v>
+      <c r="G32" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J32">
         <v>1</v>
@@ -2249,7 +2259,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A33" t="s">
         <v>17</v>
       </c>
@@ -2257,22 +2267,22 @@
         <v>17</v>
       </c>
       <c r="C33" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="D33" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="E33" t="s">
         <v>20</v>
       </c>
       <c r="F33" t="s">
-        <v>29</v>
-      </c>
-      <c r="G33" t="s">
-        <v>30</v>
-      </c>
-      <c r="H33" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J33">
         <v>1</v>
@@ -2302,7 +2312,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A34" t="s">
         <v>17</v>
       </c>
@@ -2310,19 +2320,19 @@
         <v>17</v>
       </c>
       <c r="C34" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D34" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="E34" t="s">
         <v>20</v>
       </c>
-      <c r="G34" t="s">
-        <v>21</v>
-      </c>
-      <c r="H34" t="s">
-        <v>22</v>
+      <c r="G34" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J34">
         <v>1</v>
@@ -2352,7 +2362,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A35" t="s">
         <v>17</v>
       </c>
@@ -2360,19 +2370,19 @@
         <v>17</v>
       </c>
       <c r="C35" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D35" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="E35" t="s">
         <v>20</v>
       </c>
-      <c r="G35" t="s">
-        <v>21</v>
-      </c>
-      <c r="H35" t="s">
-        <v>22</v>
+      <c r="G35" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J35">
         <v>1</v>
@@ -2402,7 +2412,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A36" t="s">
         <v>17</v>
       </c>
@@ -2410,19 +2420,19 @@
         <v>17</v>
       </c>
       <c r="C36" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D36" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="E36" t="s">
         <v>20</v>
       </c>
-      <c r="G36" t="s">
-        <v>33</v>
-      </c>
-      <c r="H36" t="s">
-        <v>34</v>
+      <c r="G36" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J36">
         <v>1</v>
@@ -2452,7 +2462,7 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A37" t="s">
         <v>17</v>
       </c>
@@ -2460,19 +2470,19 @@
         <v>17</v>
       </c>
       <c r="C37" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D37" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="E37" t="s">
         <v>20</v>
       </c>
-      <c r="G37" t="s">
-        <v>33</v>
-      </c>
-      <c r="H37" t="s">
-        <v>34</v>
+      <c r="G37" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J37">
         <v>1</v>
@@ -2502,7 +2512,7 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A38" t="s">
         <v>17</v>
       </c>
@@ -2510,19 +2520,19 @@
         <v>17</v>
       </c>
       <c r="C38" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D38" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="E38" t="s">
         <v>20</v>
       </c>
-      <c r="G38" t="s">
-        <v>33</v>
-      </c>
-      <c r="H38" t="s">
-        <v>34</v>
+      <c r="G38" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J38">
         <v>1</v>
@@ -2552,7 +2562,7 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A39" t="s">
         <v>17</v>
       </c>
@@ -2560,19 +2570,19 @@
         <v>17</v>
       </c>
       <c r="C39" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D39" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="E39" t="s">
         <v>20</v>
       </c>
-      <c r="G39" t="s">
-        <v>23</v>
-      </c>
-      <c r="H39" t="s">
-        <v>24</v>
+      <c r="G39" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J39">
         <v>1</v>
@@ -2602,7 +2612,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A40" t="s">
         <v>17</v>
       </c>
@@ -2610,19 +2620,19 @@
         <v>17</v>
       </c>
       <c r="C40" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D40" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="E40" t="s">
         <v>20</v>
       </c>
-      <c r="G40" t="s">
-        <v>23</v>
-      </c>
-      <c r="H40" t="s">
-        <v>24</v>
+      <c r="G40" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J40">
         <v>1</v>
@@ -2652,7 +2662,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A41" t="s">
         <v>17</v>
       </c>
@@ -2660,19 +2670,19 @@
         <v>17</v>
       </c>
       <c r="C41" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D41" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="E41" t="s">
         <v>20</v>
       </c>
-      <c r="G41" t="s">
-        <v>23</v>
-      </c>
-      <c r="H41" t="s">
-        <v>24</v>
+      <c r="G41" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J41">
         <v>1</v>
@@ -2702,7 +2712,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A42" t="s">
         <v>17</v>
       </c>
@@ -2710,19 +2720,19 @@
         <v>17</v>
       </c>
       <c r="C42" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="D42" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="E42" t="s">
         <v>20</v>
       </c>
-      <c r="G42" t="s">
-        <v>28</v>
-      </c>
-      <c r="H42" t="s">
-        <v>22</v>
+      <c r="G42" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H42" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J42">
         <v>1</v>
@@ -2752,7 +2762,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A43" t="s">
         <v>17</v>
       </c>
@@ -2760,19 +2770,19 @@
         <v>17</v>
       </c>
       <c r="C43" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="D43" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="E43" t="s">
         <v>20</v>
       </c>
-      <c r="G43" t="s">
-        <v>28</v>
-      </c>
-      <c r="H43" t="s">
-        <v>22</v>
+      <c r="G43" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H43" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J43">
         <v>1</v>
@@ -2802,7 +2812,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A44" t="s">
         <v>17</v>
       </c>
@@ -2810,19 +2820,19 @@
         <v>17</v>
       </c>
       <c r="C44" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="D44" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="E44" t="s">
         <v>20</v>
       </c>
-      <c r="G44" t="s">
-        <v>21</v>
-      </c>
-      <c r="H44" t="s">
-        <v>22</v>
+      <c r="G44" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J44">
         <v>1</v>
@@ -2852,7 +2862,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A45" t="s">
         <v>17</v>
       </c>
@@ -2860,19 +2870,19 @@
         <v>17</v>
       </c>
       <c r="C45" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="D45" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="E45" t="s">
         <v>20</v>
       </c>
-      <c r="G45" t="s">
-        <v>45</v>
-      </c>
-      <c r="H45" t="s">
-        <v>34</v>
+      <c r="G45" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H45" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J45">
         <v>1</v>
@@ -2902,7 +2912,7 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A46" t="s">
         <v>17</v>
       </c>
@@ -2910,22 +2920,22 @@
         <v>17</v>
       </c>
       <c r="C46" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="D46" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="E46" t="s">
         <v>20</v>
       </c>
       <c r="F46" t="s">
-        <v>29</v>
-      </c>
-      <c r="G46" t="s">
-        <v>30</v>
-      </c>
-      <c r="H46" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H46" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J46">
         <v>1</v>
@@ -2955,7 +2965,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A47" t="s">
         <v>17</v>
       </c>
@@ -2963,22 +2973,22 @@
         <v>17</v>
       </c>
       <c r="C47" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="D47" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="E47" t="s">
         <v>20</v>
       </c>
       <c r="F47" t="s">
-        <v>29</v>
-      </c>
-      <c r="G47" t="s">
-        <v>30</v>
-      </c>
-      <c r="H47" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H47" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J47">
         <v>1</v>
@@ -3008,7 +3018,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A48" t="s">
         <v>17</v>
       </c>
@@ -3016,19 +3026,19 @@
         <v>17</v>
       </c>
       <c r="C48" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="D48" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="E48" t="s">
         <v>20</v>
       </c>
-      <c r="G48" t="s">
-        <v>25</v>
-      </c>
-      <c r="H48" t="s">
-        <v>24</v>
+      <c r="G48" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H48" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J48">
         <v>1</v>
@@ -3058,27 +3068,27 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A49" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B49" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C49" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="D49" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="E49" t="s">
         <v>20</v>
       </c>
-      <c r="G49" t="s">
-        <v>28</v>
-      </c>
-      <c r="H49" t="s">
-        <v>22</v>
+      <c r="G49" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H49" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J49">
         <v>1</v>
@@ -3108,27 +3118,27 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A50" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B50" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C50" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="D50" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="E50" t="s">
         <v>20</v>
       </c>
-      <c r="G50" t="s">
-        <v>28</v>
-      </c>
-      <c r="H50" t="s">
-        <v>22</v>
+      <c r="G50" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H50" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J50">
         <v>1</v>
@@ -3158,27 +3168,27 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A51" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B51" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C51" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="D51" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="E51" t="s">
         <v>20</v>
       </c>
-      <c r="G51" t="s">
-        <v>21</v>
-      </c>
-      <c r="H51" t="s">
-        <v>22</v>
+      <c r="G51" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H51" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J51">
         <v>1</v>
@@ -3208,27 +3218,27 @@
         <v>0.23</v>
       </c>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A52" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B52" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C52" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="D52" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="E52" t="s">
         <v>20</v>
       </c>
-      <c r="G52" t="s">
-        <v>25</v>
-      </c>
-      <c r="H52" t="s">
-        <v>24</v>
+      <c r="G52" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J52">
         <v>1</v>
@@ -3258,27 +3268,27 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A53" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B53" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C53" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="D53" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="E53" t="s">
         <v>20</v>
       </c>
-      <c r="G53" t="s">
-        <v>25</v>
-      </c>
-      <c r="H53" t="s">
-        <v>24</v>
+      <c r="G53" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H53" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J53">
         <v>1</v>
@@ -3308,27 +3318,27 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A54" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B54" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C54" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="D54" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="E54" t="s">
         <v>20</v>
       </c>
-      <c r="G54" t="s">
-        <v>28</v>
-      </c>
-      <c r="H54" t="s">
-        <v>22</v>
+      <c r="G54" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J54">
         <v>1</v>
@@ -3358,27 +3368,27 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A55" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B55" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C55" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="D55" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="E55" t="s">
         <v>20</v>
       </c>
-      <c r="G55" t="s">
-        <v>21</v>
-      </c>
-      <c r="H55" t="s">
-        <v>22</v>
+      <c r="G55" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H55" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J55">
         <v>1</v>
@@ -3408,27 +3418,27 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A56" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B56" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C56" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="D56" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="E56" t="s">
         <v>20</v>
       </c>
-      <c r="G56" t="s">
-        <v>45</v>
-      </c>
-      <c r="H56" t="s">
-        <v>34</v>
+      <c r="G56" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J56">
         <v>1</v>
@@ -3458,30 +3468,30 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A57" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B57" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C57" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="D57" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="E57" t="s">
         <v>20</v>
       </c>
       <c r="F57" t="s">
-        <v>29</v>
-      </c>
-      <c r="G57" t="s">
-        <v>30</v>
-      </c>
-      <c r="H57" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H57" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J57">
         <v>1</v>
@@ -3511,30 +3521,30 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A58" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B58" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C58" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="D58" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="E58" t="s">
         <v>20</v>
       </c>
       <c r="F58" t="s">
-        <v>29</v>
-      </c>
-      <c r="G58" t="s">
-        <v>30</v>
-      </c>
-      <c r="H58" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H58" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J58">
         <v>1</v>
@@ -3564,27 +3574,27 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A59" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B59" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C59" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="D59" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="E59" t="s">
         <v>20</v>
       </c>
-      <c r="G59" t="s">
-        <v>23</v>
-      </c>
-      <c r="H59" t="s">
-        <v>24</v>
+      <c r="G59" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J59">
         <v>1</v>
@@ -3614,27 +3624,27 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A60" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B60" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C60" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="D60" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="E60" t="s">
         <v>20</v>
       </c>
-      <c r="G60" t="s">
-        <v>33</v>
-      </c>
-      <c r="H60" t="s">
-        <v>34</v>
+      <c r="G60" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H60" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J60">
         <v>1</v>
@@ -3664,27 +3674,27 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A61" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B61" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C61" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="D61" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="E61" t="s">
         <v>20</v>
       </c>
-      <c r="G61" t="s">
-        <v>33</v>
-      </c>
-      <c r="H61" t="s">
-        <v>34</v>
+      <c r="G61" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H61" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J61">
         <v>1</v>
@@ -3714,27 +3724,27 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A62" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B62" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C62" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="D62" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="E62" t="s">
         <v>20</v>
       </c>
-      <c r="G62" t="s">
-        <v>45</v>
-      </c>
-      <c r="H62" t="s">
-        <v>34</v>
+      <c r="G62" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H62" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J62">
         <v>1</v>
@@ -3764,27 +3774,27 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A63" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B63" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C63" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="D63" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="E63" t="s">
         <v>20</v>
       </c>
-      <c r="G63" t="s">
-        <v>45</v>
-      </c>
-      <c r="H63" t="s">
-        <v>34</v>
+      <c r="G63" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H63" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J63">
         <v>1</v>
@@ -3814,27 +3824,27 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A64" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B64" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C64" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="D64" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="E64" t="s">
         <v>20</v>
       </c>
-      <c r="G64" t="s">
-        <v>21</v>
-      </c>
-      <c r="H64" t="s">
-        <v>22</v>
+      <c r="G64" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H64" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J64">
         <v>1</v>
@@ -3864,30 +3874,30 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A65" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B65" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C65" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="D65" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="E65" t="s">
         <v>20</v>
       </c>
       <c r="F65" t="s">
-        <v>29</v>
-      </c>
-      <c r="G65" t="s">
-        <v>30</v>
-      </c>
-      <c r="H65" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H65" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J65">
         <v>1</v>
@@ -3917,27 +3927,27 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A66" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B66" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C66" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D66" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="E66" t="s">
-        <v>62</v>
-      </c>
-      <c r="G66" t="s">
-        <v>28</v>
-      </c>
-      <c r="H66" t="s">
-        <v>22</v>
+        <v>52</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H66" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J66">
         <v>1</v>
@@ -3967,27 +3977,27 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A67" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B67" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C67" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D67" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="E67" t="s">
-        <v>62</v>
-      </c>
-      <c r="G67" t="s">
-        <v>21</v>
-      </c>
-      <c r="H67" t="s">
-        <v>22</v>
+        <v>52</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H67" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J67">
         <v>1</v>
@@ -4017,27 +4027,27 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A68" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B68" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C68" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D68" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="E68" t="s">
-        <v>62</v>
-      </c>
-      <c r="G68" t="s">
-        <v>23</v>
-      </c>
-      <c r="H68" t="s">
-        <v>24</v>
+        <v>52</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H68" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J68">
         <v>1</v>
@@ -4067,27 +4077,27 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A69" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B69" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C69" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D69" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="E69" t="s">
-        <v>62</v>
-      </c>
-      <c r="G69" t="s">
-        <v>23</v>
-      </c>
-      <c r="H69" t="s">
-        <v>24</v>
+        <v>52</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H69" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J69">
         <v>1</v>
@@ -4117,27 +4127,27 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A70" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B70" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C70" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="D70" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E70" t="s">
         <v>20</v>
       </c>
-      <c r="G70" t="s">
-        <v>21</v>
-      </c>
-      <c r="H70" t="s">
-        <v>22</v>
+      <c r="G70" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H70" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J70">
         <v>1</v>
@@ -4167,27 +4177,27 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A71" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B71" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C71" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="D71" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E71" t="s">
         <v>20</v>
       </c>
-      <c r="G71" t="s">
-        <v>21</v>
-      </c>
-      <c r="H71" t="s">
-        <v>22</v>
+      <c r="G71" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H71" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J71">
         <v>1</v>
@@ -4217,27 +4227,27 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A72" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B72" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C72" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="D72" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E72" t="s">
         <v>20</v>
       </c>
-      <c r="G72" t="s">
-        <v>33</v>
-      </c>
-      <c r="H72" t="s">
-        <v>34</v>
+      <c r="G72" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J72">
         <v>1</v>
@@ -4267,27 +4277,27 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A73" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B73" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C73" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="D73" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E73" t="s">
         <v>20</v>
       </c>
-      <c r="G73" t="s">
-        <v>33</v>
-      </c>
-      <c r="H73" t="s">
-        <v>34</v>
+      <c r="G73" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H73" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J73">
         <v>1</v>
@@ -4317,27 +4327,27 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A74" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B74" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C74" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="D74" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E74" t="s">
         <v>20</v>
       </c>
-      <c r="G74" t="s">
-        <v>25</v>
-      </c>
-      <c r="H74" t="s">
-        <v>24</v>
+      <c r="G74" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H74" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J74">
         <v>1</v>
@@ -4367,27 +4377,27 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A75" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B75" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C75" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="D75" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E75" t="s">
         <v>20</v>
       </c>
-      <c r="G75" t="s">
-        <v>23</v>
-      </c>
-      <c r="H75" t="s">
-        <v>24</v>
+      <c r="G75" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H75" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J75">
         <v>1</v>
@@ -4417,30 +4427,30 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A76" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B76" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C76" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="D76" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E76" t="s">
         <v>20</v>
       </c>
       <c r="F76" t="s">
-        <v>29</v>
-      </c>
-      <c r="G76" t="s">
-        <v>30</v>
-      </c>
-      <c r="H76" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H76" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J76">
         <v>1</v>
@@ -4470,30 +4480,30 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="77" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A77" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B77" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C77" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="D77" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E77" t="s">
         <v>20</v>
       </c>
       <c r="F77" t="s">
-        <v>29</v>
-      </c>
-      <c r="G77" t="s">
-        <v>30</v>
-      </c>
-      <c r="H77" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H77" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J77">
         <v>1</v>
@@ -4523,27 +4533,27 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="78" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A78" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B78" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C78" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D78" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="E78" t="s">
-        <v>62</v>
-      </c>
-      <c r="G78" t="s">
-        <v>28</v>
-      </c>
-      <c r="H78" t="s">
-        <v>22</v>
+        <v>52</v>
+      </c>
+      <c r="G78" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H78" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J78">
         <v>1</v>
@@ -4573,27 +4583,27 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="79" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A79" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B79" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C79" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D79" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="E79" t="s">
-        <v>62</v>
-      </c>
-      <c r="G79" t="s">
-        <v>28</v>
-      </c>
-      <c r="H79" t="s">
-        <v>22</v>
+        <v>52</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H79" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J79">
         <v>1</v>
@@ -4623,27 +4633,27 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="80" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A80" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B80" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C80" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D80" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="E80" t="s">
-        <v>62</v>
-      </c>
-      <c r="G80" t="s">
-        <v>23</v>
-      </c>
-      <c r="H80" t="s">
-        <v>24</v>
+        <v>52</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H80" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J80">
         <v>1</v>
@@ -4673,27 +4683,27 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A81" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="B81" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C81" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D81" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="E81" t="s">
-        <v>62</v>
-      </c>
-      <c r="G81" t="s">
-        <v>23</v>
-      </c>
-      <c r="H81" t="s">
-        <v>24</v>
+        <v>52</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H81" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J81">
         <v>1</v>
@@ -4723,27 +4733,27 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A82" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B82" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C82" t="s">
+        <v>58</v>
+      </c>
+      <c r="D82" t="s">
+        <v>59</v>
+      </c>
+      <c r="E82" t="s">
+        <v>52</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H82" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="D82" t="s">
-        <v>69</v>
-      </c>
-      <c r="E82" t="s">
-        <v>62</v>
-      </c>
-      <c r="G82" t="s">
-        <v>28</v>
-      </c>
-      <c r="H82" t="s">
-        <v>22</v>
       </c>
       <c r="J82">
         <v>1</v>
@@ -4773,27 +4783,27 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A83" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B83" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C83" t="s">
+        <v>58</v>
+      </c>
+      <c r="D83" t="s">
+        <v>59</v>
+      </c>
+      <c r="E83" t="s">
+        <v>52</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H83" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="D83" t="s">
-        <v>69</v>
-      </c>
-      <c r="E83" t="s">
-        <v>62</v>
-      </c>
-      <c r="G83" t="s">
-        <v>33</v>
-      </c>
-      <c r="H83" t="s">
-        <v>34</v>
       </c>
       <c r="J83">
         <v>1</v>
@@ -4823,27 +4833,27 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A84" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B84" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C84" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="D84" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="E84" t="s">
-        <v>62</v>
-      </c>
-      <c r="G84" t="s">
-        <v>25</v>
-      </c>
-      <c r="H84" t="s">
-        <v>24</v>
+        <v>52</v>
+      </c>
+      <c r="G84" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H84" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J84">
         <v>1</v>
@@ -4873,30 +4883,30 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A85" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B85" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C85" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="D85" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="E85" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="F85" t="s">
-        <v>29</v>
-      </c>
-      <c r="G85" t="s">
-        <v>30</v>
-      </c>
-      <c r="H85" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H85" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J85">
         <v>1</v>
@@ -4926,27 +4936,27 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A86" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B86" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C86" t="s">
+        <v>60</v>
+      </c>
+      <c r="D86" t="s">
+        <v>61</v>
+      </c>
+      <c r="E86" t="s">
+        <v>20</v>
+      </c>
+      <c r="G86" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D86" t="s">
-        <v>71</v>
-      </c>
-      <c r="E86" t="s">
-        <v>20</v>
-      </c>
-      <c r="G86" t="s">
-        <v>33</v>
-      </c>
-      <c r="H86" t="s">
-        <v>34</v>
+      <c r="H86" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J86">
         <v>1</v>
@@ -4976,27 +4986,27 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A87" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B87" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C87" t="s">
+        <v>60</v>
+      </c>
+      <c r="D87" t="s">
+        <v>61</v>
+      </c>
+      <c r="E87" t="s">
+        <v>20</v>
+      </c>
+      <c r="G87" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D87" t="s">
-        <v>71</v>
-      </c>
-      <c r="E87" t="s">
-        <v>20</v>
-      </c>
-      <c r="G87" t="s">
-        <v>33</v>
-      </c>
-      <c r="H87" t="s">
-        <v>34</v>
+      <c r="H87" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J87">
         <v>1</v>
@@ -5026,27 +5036,27 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A88" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B88" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C88" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D88" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="E88" t="s">
         <v>20</v>
       </c>
-      <c r="G88" t="s">
-        <v>45</v>
-      </c>
-      <c r="H88" t="s">
-        <v>34</v>
+      <c r="G88" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H88" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J88">
         <v>1</v>
@@ -5076,27 +5086,27 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A89" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B89" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C89" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D89" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="E89" t="s">
         <v>20</v>
       </c>
-      <c r="G89" t="s">
-        <v>45</v>
-      </c>
-      <c r="H89" t="s">
-        <v>34</v>
+      <c r="G89" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H89" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="J89">
         <v>1</v>
@@ -5126,27 +5136,27 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A90" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B90" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C90" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="D90" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="E90" t="s">
         <v>20</v>
       </c>
-      <c r="G90" t="s">
-        <v>28</v>
-      </c>
-      <c r="H90" t="s">
-        <v>22</v>
+      <c r="G90" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H90" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J90">
         <v>1</v>
@@ -5176,27 +5186,27 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A91" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B91" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C91" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="D91" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="E91" t="s">
         <v>20</v>
       </c>
-      <c r="G91" t="s">
-        <v>28</v>
-      </c>
-      <c r="H91" t="s">
-        <v>22</v>
+      <c r="G91" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H91" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J91">
         <v>1</v>
@@ -5226,27 +5236,27 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A92" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B92" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C92" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="D92" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="E92" t="s">
         <v>20</v>
       </c>
-      <c r="G92" t="s">
-        <v>23</v>
-      </c>
-      <c r="H92" t="s">
-        <v>24</v>
+      <c r="G92" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H92" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J92">
         <v>1</v>
@@ -5276,27 +5286,27 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A93" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B93" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C93" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="D93" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="E93" t="s">
         <v>20</v>
       </c>
-      <c r="G93" t="s">
-        <v>23</v>
-      </c>
-      <c r="H93" t="s">
-        <v>24</v>
+      <c r="G93" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H93" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J93">
         <v>1</v>
@@ -5326,27 +5336,27 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A94" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B94" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C94" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="D94" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E94" t="s">
-        <v>62</v>
-      </c>
-      <c r="G94" t="s">
-        <v>21</v>
-      </c>
-      <c r="H94" t="s">
-        <v>22</v>
+        <v>52</v>
+      </c>
+      <c r="G94" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H94" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J94">
         <v>1</v>
@@ -5376,27 +5386,27 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A95" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B95" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C95" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="D95" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E95" t="s">
-        <v>62</v>
-      </c>
-      <c r="G95" t="s">
-        <v>33</v>
-      </c>
-      <c r="H95" t="s">
-        <v>34</v>
+        <v>52</v>
+      </c>
+      <c r="G95" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H95" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J95">
         <v>1</v>
@@ -5426,27 +5436,27 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A96" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B96" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C96" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="D96" t="s">
+        <v>65</v>
+      </c>
+      <c r="E96" t="s">
+        <v>52</v>
+      </c>
+      <c r="G96" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="H96" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="E96" t="s">
-        <v>62</v>
-      </c>
-      <c r="G96" t="s">
-        <v>45</v>
-      </c>
-      <c r="H96" t="s">
-        <v>34</v>
       </c>
       <c r="J96">
         <v>1</v>
@@ -5476,27 +5486,27 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="97" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A97" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B97" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C97" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="D97" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E97" t="s">
-        <v>62</v>
-      </c>
-      <c r="G97" t="s">
-        <v>23</v>
-      </c>
-      <c r="H97" t="s">
-        <v>24</v>
+        <v>52</v>
+      </c>
+      <c r="G97" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H97" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="J97">
         <v>1</v>
@@ -5526,27 +5536,27 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="98" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A98" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B98" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C98" t="s">
+        <v>64</v>
+      </c>
+      <c r="D98" t="s">
+        <v>65</v>
+      </c>
+      <c r="E98" t="s">
+        <v>52</v>
+      </c>
+      <c r="G98" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D98" t="s">
-        <v>75</v>
-      </c>
-      <c r="E98" t="s">
-        <v>62</v>
-      </c>
-      <c r="G98" t="s">
-        <v>25</v>
-      </c>
-      <c r="H98" t="s">
-        <v>24</v>
+      <c r="H98" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="J98">
         <v>1</v>
@@ -5576,30 +5586,30 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="99" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:19" x14ac:dyDescent="0.8">
       <c r="A99" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B99" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C99" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="D99" t="s">
+        <v>65</v>
+      </c>
+      <c r="E99" t="s">
+        <v>52</v>
+      </c>
+      <c r="F99" t="s">
+        <v>23</v>
+      </c>
+      <c r="G99" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H99" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="E99" t="s">
-        <v>62</v>
-      </c>
-      <c r="F99" t="s">
-        <v>29</v>
-      </c>
-      <c r="G99" t="s">
-        <v>30</v>
-      </c>
-      <c r="H99" t="s">
-        <v>24</v>
       </c>
       <c r="J99">
         <v>1</v>

</xml_diff>